<commit_message>
refactor: Enhance expedition flow and introduce new condition configurations
- Added new condition configurations for expedition flow, including CounterAtLeastConditionConfig, HasFlagConditionConfig, HasItemConditionConfig, and HasChosenOptionConditionConfig.
- Introduced EnumExpeditionRoutePolicy to manage route policies within expedition nodes.
- Updated ExpeditionRouteNodeConfig to incorporate new properties for route policies and transitions.
- Enhanced ExpeditionFlowController with methods for managing blackboard flags, items, and counters, improving dynamic node insertion capabilities.
- Refactored existing gameplay logic to accommodate new configurations and streamline expedition flow management.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>##var</t>
   </si>
@@ -58,6 +58,30 @@
     <t>combat_encounter_id</t>
   </si>
   <si>
+    <t>route_policy</t>
+  </si>
+  <si>
+    <t>default_transition_id</t>
+  </si>
+  <si>
+    <t>*transitions</t>
+  </si>
+  <si>
+    <t>option_routes</t>
+  </si>
+  <si>
+    <t>transition_id</t>
+  </si>
+  <si>
+    <t>target_node_id</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>conditions</t>
+  </si>
+  <si>
     <t>##type</t>
   </si>
   <si>
@@ -74,6 +98,12 @@
   </si>
   <si>
     <t>废墟补给点</t>
+  </si>
+  <si>
+    <t>fixed_next</t>
+  </si>
+  <si>
+    <t>1,1</t>
   </si>
   <si>
     <t>Combat</t>
@@ -465,7 +495,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -480,6 +510,30 @@
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -625,7 +679,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
@@ -637,34 +691,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0">
@@ -749,7 +803,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -768,23 +822,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1118,199 +1169,267 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.2727272727273" style="6" customWidth="1"/>
-    <col min="4" max="4" width="26.3636363636364" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15.2727272727273" style="6" customWidth="1"/>
-    <col min="6" max="6" width="11.5454545454545" style="6" customWidth="1"/>
-    <col min="7" max="7" width="12.2727272727273" style="6" customWidth="1"/>
-    <col min="8" max="8" width="23.8181818181818" style="6" customWidth="1"/>
-    <col min="9" max="14" width="9" style="6"/>
+    <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
+    <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
+    <col min="5" max="5" width="15.2727272727273" style="5" customWidth="1"/>
+    <col min="6" max="6" width="11.5454545454545" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.2727272727273" style="5" customWidth="1"/>
+    <col min="8" max="8" width="23.8181818181818" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.2727272727273" style="5" customWidth="1"/>
+    <col min="10" max="10" width="26.2727272727273" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="12" max="12" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="13" max="14" width="14" style="5" customWidth="1"/>
+    <col min="15" max="15" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="16" max="17" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:14">
-      <c r="A1" s="7" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:17">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="11"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
       <c r="N1" s="9"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:14">
-      <c r="A2" s="7" t="s">
+    <row r="2" s="1" customFormat="1" spans="1:17">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
+      <c r="I2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="L2" s="9"/>
       <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:14">
-      <c r="A3" s="7" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:17">
+      <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:14">
-      <c r="A4" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
+    <row r="4" s="2" customFormat="1" spans="1:17">
+      <c r="A4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:14">
-      <c r="A5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
+    <row r="5" s="3" customFormat="1" spans="1:17">
+      <c r="A5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:14">
-      <c r="A6" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
+    <row r="6" s="3" customFormat="1" spans="1:17">
+      <c r="A6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:14">
-      <c r="A7" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:17">
+      <c r="A7" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="15"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
     </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="6">
+    <row r="8" spans="1:17">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="5">
         <v>1</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>14</v>
+      <c r="F8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="5">
+        <v>1</v>
+      </c>
+      <c r="K8" s="5">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5">
+        <v>2</v>
+      </c>
+      <c r="M8" s="5">
+        <v>1</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="E9" s="6">
+    <row r="9" spans="1:17">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="E9" s="5">
         <v>2</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>16</v>
+      <c r="F9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="E1:H1"/>
+  <mergeCells count="2">
+    <mergeCell ref="E1:O1"/>
+    <mergeCell ref="K2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
refactor: Update expedition configuration identifiers and streamline data handling
- Renamed various identifiers in expedition configuration files to use "config_id" suffix for consistency and clarity.
- Updated related JSON files to reflect changes in identifier naming conventions, enhancing data integrity.
- Refactored gameplay logic to accommodate new identifier names, improving readability and maintainability across expedition flow and combat session handling.
- Ensured all references to identifiers are consistent throughout the codebase, reducing potential errors and improving overall code quality.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -34,7 +34,7 @@
     <t>##var</t>
   </si>
   <si>
-    <t>expedition_id</t>
+    <t>expedition_config_id</t>
   </si>
   <si>
     <t>name</t>
@@ -46,16 +46,16 @@
     <t>*route</t>
   </si>
   <si>
-    <t>node_id</t>
+    <t>node_config_id</t>
   </si>
   <si>
     <t>node_type</t>
   </si>
   <si>
-    <t>event_id</t>
-  </si>
-  <si>
-    <t>combat_encounter_id</t>
+    <t>event_config_id</t>
+  </si>
+  <si>
+    <t>combat_encounter_config_id</t>
   </si>
   <si>
     <t>route_policy</t>
@@ -73,7 +73,7 @@
     <t>transition_id</t>
   </si>
   <si>
-    <t>target_node_id</t>
+    <t>target_node_config_id</t>
   </si>
   <si>
     <t>priority</t>
@@ -1173,17 +1173,17 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
-    <col min="2" max="2" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
     <col min="5" max="5" width="15.2727272727273" style="5" customWidth="1"/>
     <col min="6" max="6" width="11.5454545454545" style="5" customWidth="1"/>
-    <col min="7" max="7" width="12.2727272727273" style="5" customWidth="1"/>
+    <col min="7" max="7" width="18.9090909090909" style="5" customWidth="1"/>
     <col min="8" max="8" width="23.8181818181818" style="5" customWidth="1"/>
     <col min="9" max="9" width="15.2727272727273" style="5" customWidth="1"/>
     <col min="10" max="10" width="26.2727272727273" style="5" customWidth="1"/>
     <col min="11" max="11" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="12" max="12" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="12" max="12" width="26.2727272727273" style="5" customWidth="1"/>
     <col min="13" max="14" width="14" style="5" customWidth="1"/>
     <col min="15" max="15" width="16.4545454545455" style="5" customWidth="1"/>
     <col min="16" max="17" width="9" style="5"/>

</xml_diff>

<commit_message>
refactor: Update expedition configuration files and streamline data structures
- Modified expedition configuration files, removing the default_transition_id field to simplify data structures.
- Updated related JSON files to reflect changes in node transition handling, enhancing clarity and maintainability.
- Refactored gameplay logic to accommodate new data structures, improving readability and consistency across expedition flow.
- Ensured all references to identifiers and configurations are consistent throughout the codebase, reducing potential errors.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>##var</t>
   </si>
@@ -61,9 +61,6 @@
     <t>route_policy</t>
   </si>
   <si>
-    <t>default_transition_id</t>
-  </si>
-  <si>
     <t>*transitions</t>
   </si>
   <si>
@@ -85,6 +82,24 @@
     <t>##type</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>EnumExpeditionNodeType</t>
+  </si>
+  <si>
+    <t>EnumExpeditionRoutePolicy</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>list, ExpeditionNodeTransitionConfig</t>
+  </si>
+  <si>
+    <t>list, ExpeditionOptionRouteConfig</t>
+  </si>
+  <si>
     <t>##</t>
   </si>
   <si>
@@ -94,7 +109,7 @@
     <t>附加的森林，不算太危险</t>
   </si>
   <si>
-    <t>Event</t>
+    <t>event</t>
   </si>
   <si>
     <t>废墟补给点</t>
@@ -103,10 +118,7 @@
     <t>fixed_next</t>
   </si>
   <si>
-    <t>1,1</t>
-  </si>
-  <si>
-    <t>Combat</t>
+    <t>combat</t>
   </si>
   <si>
     <t>前哨遭遇战</t>
@@ -1169,27 +1181,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
-    <col min="5" max="5" width="15.2727272727273" style="5" customWidth="1"/>
-    <col min="6" max="6" width="11.5454545454545" style="5" customWidth="1"/>
+    <col min="5" max="5" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.5454545454545" style="5" customWidth="1"/>
     <col min="7" max="7" width="18.9090909090909" style="5" customWidth="1"/>
     <col min="8" max="8" width="23.8181818181818" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.2727272727273" style="5" customWidth="1"/>
-    <col min="10" max="10" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="11" max="11" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="12" max="12" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="13" max="14" width="14" style="5" customWidth="1"/>
-    <col min="15" max="15" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="16" max="17" width="9" style="5"/>
+    <col min="9" max="9" width="31.1818181818182" style="5" customWidth="1"/>
+    <col min="10" max="10" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="11" max="11" width="26.2727272727273" style="5" customWidth="1"/>
+    <col min="12" max="13" width="14" style="5" customWidth="1"/>
+    <col min="14" max="14" width="41" style="5" customWidth="1"/>
+    <col min="15" max="16" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:17">
+    <row r="1" s="1" customFormat="1" spans="1:16">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1213,12 +1224,11 @@
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="7"/>
       <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:17">
+    <row r="2" s="1" customFormat="1" spans="1:16">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -1240,22 +1250,19 @@
       <c r="I2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="O2" s="7"/>
       <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:17">
+    <row r="3" s="1" customFormat="1" spans="1:16">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1267,7 +1274,9 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="K3" s="7" t="s">
         <v>13</v>
       </c>
@@ -1277,37 +1286,59 @@
       <c r="M3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:17">
+    <row r="4" s="2" customFormat="1" spans="1:16">
       <c r="A4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="12"/>
+      <c r="C4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="O4" s="12"/>
       <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:17">
+    <row r="5" s="3" customFormat="1" spans="1:16">
       <c r="A5" s="13" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
@@ -1324,11 +1355,10 @@
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
       <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:17">
+    <row r="6" s="3" customFormat="1" spans="1:16">
       <c r="A6" s="13" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
@@ -1345,11 +1375,10 @@
       <c r="N6" s="14"/>
       <c r="O6" s="14"/>
       <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:17">
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:16">
       <c r="A7" s="15" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="16"/>
@@ -1366,70 +1395,63 @@
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
       <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:16">
       <c r="A8" s="17"/>
       <c r="B8" s="17" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="J8" s="5">
         <v>1</v>
       </c>
       <c r="K8" s="5">
-        <v>1</v>
-      </c>
-      <c r="L8" s="5">
         <v>2</v>
       </c>
-      <c r="M8" s="5">
-        <v>1</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:16">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="E9" s="5">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="J9" s="5">
+        <v>1</v>
+      </c>
+      <c r="K9" s="5">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E1:O1"/>
-    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="J2:M2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
refactor: Enhance expedition configuration and random event handling
- Updated expedition XML and JSON files to introduce new random event configurations and environment settings.
- Added support for random events in the expedition flow, allowing for dynamic gameplay experiences.
- Refactored related classes to accommodate new configurations, improving clarity and maintainability.
- Enhanced combat session handling to integrate battlefield configurations, ensuring a cohesive gameplay experience.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
   <si>
     <t>##var</t>
   </si>
@@ -43,6 +43,12 @@
     <t>description</t>
   </si>
   <si>
+    <t>initial_environment_config_id</t>
+  </si>
+  <si>
+    <t>lst_random_event_pool_config_id</t>
+  </si>
+  <si>
     <t>*route</t>
   </si>
   <si>
@@ -85,6 +91,9 @@
     <t>string</t>
   </si>
   <si>
+    <t>list,string</t>
+  </si>
+  <si>
     <t>EnumExpeditionNodeType</t>
   </si>
   <si>
@@ -109,6 +118,9 @@
     <t>附加的森林，不算太危险</t>
   </si>
   <si>
+    <t>普通森林</t>
+  </si>
+  <si>
     <t>event</t>
   </si>
   <si>
@@ -116,6 +128,9 @@
   </si>
   <si>
     <t>fixed_next</t>
+  </si>
+  <si>
+    <t>random_event</t>
   </si>
   <si>
     <t>combat</t>
@@ -815,7 +830,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -838,6 +853,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1181,26 +1199,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
     <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
-    <col min="5" max="5" width="17.7272727272727" style="5" customWidth="1"/>
-    <col min="6" max="6" width="27.5454545454545" style="5" customWidth="1"/>
-    <col min="7" max="7" width="18.9090909090909" style="5" customWidth="1"/>
-    <col min="8" max="8" width="23.8181818181818" style="5" customWidth="1"/>
-    <col min="9" max="9" width="31.1818181818182" style="5" customWidth="1"/>
-    <col min="10" max="10" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="11" max="11" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="12" max="13" width="14" style="5" customWidth="1"/>
-    <col min="14" max="14" width="41" style="5" customWidth="1"/>
-    <col min="15" max="16" width="9" style="5"/>
+    <col min="5" max="6" width="36.0909090909091" style="5" customWidth="1"/>
+    <col min="7" max="7" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="8" max="8" width="27.5454545454545" style="5" customWidth="1"/>
+    <col min="9" max="9" width="18.9090909090909" style="5" customWidth="1"/>
+    <col min="10" max="10" width="23.8181818181818" style="5" customWidth="1"/>
+    <col min="11" max="11" width="31.1818181818182" style="5" customWidth="1"/>
+    <col min="12" max="12" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="13" max="13" width="26.2727272727273" style="5" customWidth="1"/>
+    <col min="14" max="15" width="14" style="5" customWidth="1"/>
+    <col min="16" max="16" width="41" style="5" customWidth="1"/>
+    <col min="17" max="18" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:16">
+    <row r="1" s="1" customFormat="1" spans="1:18">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1216,31 +1235,33 @@
       <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
+      <c r="F1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
       <c r="N1" s="10"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:16">
+    <row r="2" s="1" customFormat="1" spans="1:18">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
-      <c r="E2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>6</v>
-      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
       <c r="G2" s="7" t="s">
         <v>7</v>
       </c>
@@ -1250,19 +1271,25 @@
       <c r="I2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
+      <c r="K2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="M2" s="10"/>
-      <c r="N2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:16">
+    <row r="3" s="1" customFormat="1" spans="1:18">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1274,184 +1301,220 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>13</v>
-      </c>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
       <c r="L3" s="7" t="s">
         <v>14</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
+      <c r="N3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:16">
-      <c r="A4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="12" t="s">
+    <row r="4" s="2" customFormat="1" spans="1:18">
+      <c r="A4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="12" t="s">
+      <c r="B4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="L4" s="12" t="s">
+      <c r="C4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="G4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="I4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
+      <c r="L4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="13"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:16">
-      <c r="A5" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
+    <row r="5" s="3" customFormat="1" spans="1:18">
+      <c r="A5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:16">
-      <c r="A6" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
+    <row r="6" s="3" customFormat="1" spans="1:18">
+      <c r="A6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:16">
-      <c r="A7" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:18">
+      <c r="A7" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
     </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="5">
+    <row r="8" spans="1:18">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8" s="5">
         <v>1</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="J8" s="5">
+      <c r="H8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L8" s="5">
         <v>1</v>
       </c>
-      <c r="K8" s="5">
+      <c r="M8" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="E9" s="5">
+    <row r="9" spans="1:18">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="5">
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="J9" s="5">
+      <c r="H9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="18"/>
+      <c r="K9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L9" s="5">
         <v>1</v>
       </c>
-      <c r="K9" s="5">
-        <v>1</v>
+      <c r="M9" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="G10" s="5">
+        <v>3</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E1:N1"/>
-    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="G1:P1"/>
+    <mergeCell ref="L2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Introduce expedition reward profile system and enhance reward handling
- Added new expedition reward profile configuration to define rewards across different stages and tiers.
- Updated expedition XML and JSON files to integrate reward profiles, allowing for dynamic reward allocation during expeditions.
- Enhanced existing effects (AddMoneyEffect, AddPlayerMarbleExpEffect, AddPlayerMarbleHpEffect) to utilize the new reward profile system for calculating rewards based on progress stages and tiers.
- Refactored ExpeditionEffectExecutionContext and related classes to support the new reward context, improving the overall expedition flow and reward management.
- Implemented logging for missing configurations to aid in debugging and ensure robust gameplay experiences.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
   <si>
     <t>##var</t>
   </si>
@@ -43,6 +43,9 @@
     <t>description</t>
   </si>
   <si>
+    <t>reward_profile_config_id</t>
+  </si>
+  <si>
     <t>initial_environment_config_id</t>
   </si>
   <si>
@@ -116,6 +119,9 @@
   </si>
   <si>
     <t>附加的森林，不算太危险</t>
+  </si>
+  <si>
+    <t>配置1</t>
   </si>
   <si>
     <t>普通森林</t>
@@ -830,7 +836,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -853,6 +859,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1199,27 +1208,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
-    <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
-    <col min="5" max="6" width="36.0909090909091" style="5" customWidth="1"/>
-    <col min="7" max="7" width="17.7272727272727" style="5" customWidth="1"/>
-    <col min="8" max="8" width="27.5454545454545" style="5" customWidth="1"/>
-    <col min="9" max="9" width="18.9090909090909" style="5" customWidth="1"/>
-    <col min="10" max="10" width="23.8181818181818" style="5" customWidth="1"/>
-    <col min="11" max="11" width="31.1818181818182" style="5" customWidth="1"/>
-    <col min="12" max="12" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="13" max="13" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="14" max="15" width="14" style="5" customWidth="1"/>
-    <col min="16" max="16" width="41" style="5" customWidth="1"/>
-    <col min="17" max="18" width="9" style="5"/>
+    <col min="4" max="5" width="26.3636363636364" style="5" customWidth="1"/>
+    <col min="6" max="7" width="36.0909090909091" style="5" customWidth="1"/>
+    <col min="8" max="8" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="9" max="9" width="27.5454545454545" style="5" customWidth="1"/>
+    <col min="10" max="10" width="18.9090909090909" style="5" customWidth="1"/>
+    <col min="11" max="11" width="23.8181818181818" style="5" customWidth="1"/>
+    <col min="12" max="12" width="31.1818181818182" style="5" customWidth="1"/>
+    <col min="13" max="13" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="14" max="14" width="26.2727272727273" style="5" customWidth="1"/>
+    <col min="15" max="16" width="14" style="5" customWidth="1"/>
+    <col min="17" max="17" width="41" style="5" customWidth="1"/>
+    <col min="18" max="19" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:18">
+    <row r="1" s="1" customFormat="1" spans="1:19">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1235,25 +1244,28 @@
       <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
+      <c r="H1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
       <c r="P1" s="11"/>
-      <c r="Q1" s="7"/>
+      <c r="Q1" s="12"/>
       <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:18">
+    <row r="2" s="1" customFormat="1" spans="1:19">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -1262,9 +1274,7 @@
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
-      <c r="G2" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="G2" s="7"/>
       <c r="H2" s="7" t="s">
         <v>8</v>
       </c>
@@ -1277,19 +1287,22 @@
       <c r="K2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
+      <c r="M2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="11"/>
       <c r="O2" s="11"/>
-      <c r="P2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="7"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="7" t="s">
+        <v>14</v>
+      </c>
       <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:18">
+    <row r="3" s="1" customFormat="1" spans="1:19">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1303,9 +1316,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="7" t="s">
-        <v>14</v>
-      </c>
+      <c r="L3" s="7"/>
       <c r="M3" s="7" t="s">
         <v>15</v>
       </c>
@@ -1315,206 +1326,219 @@
       <c r="O3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="7"/>
+      <c r="P3" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:18">
-      <c r="A4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="12" t="s">
+    <row r="4" s="2" customFormat="1" spans="1:19">
+      <c r="A4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="13" t="s">
+      <c r="B4" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="13" t="s">
+      <c r="C4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="13" t="s">
+      <c r="H4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="N4" s="13" t="s">
+      <c r="J4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="M4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="P4" s="13" t="s">
+      <c r="P4" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
+      <c r="Q4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" s="14"/>
+      <c r="S4" s="14"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:18">
-      <c r="A5" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
+    <row r="5" s="3" customFormat="1" spans="1:19">
+      <c r="A5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:18">
-      <c r="A6" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
+    <row r="6" s="3" customFormat="1" spans="1:19">
+      <c r="A6" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:18">
-      <c r="A7" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
-      <c r="R7" s="17"/>
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:19">
+      <c r="A7" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
     </row>
-    <row r="8" spans="1:18">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="18" t="s">
+    <row r="8" spans="1:19">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="C8" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="5">
+      <c r="E8" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="19"/>
+      <c r="H8" s="5">
         <v>1</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="K8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="L8" s="5">
+      <c r="J8" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M8" s="5">
         <v>1</v>
       </c>
-      <c r="M8" s="5">
+      <c r="N8" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:18">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="5">
+    <row r="9" spans="1:19">
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="5">
         <v>2</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="18"/>
-      <c r="K9" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="L9" s="5">
+      <c r="I9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="L9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M9" s="5">
         <v>1</v>
       </c>
-      <c r="M9" s="5">
+      <c r="N9" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:18">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-      <c r="G10" s="5">
+    <row r="10" spans="1:19">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="H10" s="5">
         <v>3</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="I10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="J10" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="G1:P1"/>
-    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="H1:Q1"/>
+    <mergeCell ref="M2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Enhance expedition configurations with enemy profiles and dynamic enemy handling
- Introduced new enemy profile configuration to define enemy counts and levels across different stages of expeditions.
- Updated XML and JSON files to integrate enemy profiles, allowing for dynamic enemy generation based on environment candidates and enemy profiles.
- Enhanced combat encounter configurations to support dynamic enemy groups, improving gameplay dynamics and challenge.
- Refactored related classes to utilize the new enemy profile system, ensuring cohesive integration within the expedition flow.
- Improved documentation and comments to clarify the new enemy handling mechanics and their impact on gameplay.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition.xlsx
+++ b/Configs/GameConfig/Datas/expedition.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
     <t>##var</t>
   </si>
@@ -46,6 +46,9 @@
     <t>reward_profile_config_id</t>
   </si>
   <si>
+    <t>enemy_profile_config_id</t>
+  </si>
+  <si>
     <t>initial_environment_config_id</t>
   </si>
   <si>
@@ -121,7 +124,10 @@
     <t>附加的森林，不算太危险</t>
   </si>
   <si>
-    <t>配置1</t>
+    <t>奖励配置1</t>
+  </si>
+  <si>
+    <t>敌人配置1</t>
   </si>
   <si>
     <t>普通森林</t>
@@ -836,7 +842,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -859,9 +865,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1208,27 +1211,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
-    <col min="4" max="5" width="26.3636363636364" style="5" customWidth="1"/>
-    <col min="6" max="7" width="36.0909090909091" style="5" customWidth="1"/>
-    <col min="8" max="8" width="17.7272727272727" style="5" customWidth="1"/>
-    <col min="9" max="9" width="27.5454545454545" style="5" customWidth="1"/>
-    <col min="10" max="10" width="18.9090909090909" style="5" customWidth="1"/>
-    <col min="11" max="11" width="23.8181818181818" style="5" customWidth="1"/>
-    <col min="12" max="12" width="31.1818181818182" style="5" customWidth="1"/>
-    <col min="13" max="13" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="14" max="14" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="15" max="16" width="14" style="5" customWidth="1"/>
-    <col min="17" max="17" width="41" style="5" customWidth="1"/>
-    <col min="18" max="19" width="9" style="5"/>
+    <col min="4" max="4" width="26.3636363636364" style="5" customWidth="1"/>
+    <col min="5" max="5" width="30" style="5" customWidth="1"/>
+    <col min="6" max="6" width="26.3636363636364" style="5" customWidth="1"/>
+    <col min="7" max="8" width="36.0909090909091" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="10" max="10" width="27.5454545454545" style="5" customWidth="1"/>
+    <col min="11" max="11" width="18.9090909090909" style="5" customWidth="1"/>
+    <col min="12" max="12" width="23.8181818181818" style="5" customWidth="1"/>
+    <col min="13" max="13" width="31.1818181818182" style="5" customWidth="1"/>
+    <col min="14" max="14" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="15" max="15" width="26.2727272727273" style="5" customWidth="1"/>
+    <col min="16" max="17" width="14" style="5" customWidth="1"/>
+    <col min="18" max="18" width="41" style="5" customWidth="1"/>
+    <col min="19" max="20" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:19">
+    <row r="1" s="1" customFormat="1" spans="1:20">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1244,28 +1249,31 @@
       <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="7"/>
+      <c r="I1" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="11"/>
       <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:19">
+    <row r="2" s="1" customFormat="1" spans="1:20">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -1275,9 +1283,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
-      <c r="H2" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="H2" s="7"/>
       <c r="I2" s="7" t="s">
         <v>9</v>
       </c>
@@ -1290,19 +1296,22 @@
       <c r="L2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="7" t="s">
+      <c r="N2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="7"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:19">
+    <row r="3" s="1" customFormat="1" spans="1:20">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1317,9 +1326,7 @@
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
-      <c r="M3" s="7" t="s">
-        <v>15</v>
-      </c>
+      <c r="M3" s="7"/>
       <c r="N3" s="7" t="s">
         <v>16</v>
       </c>
@@ -1329,216 +1336,227 @@
       <c r="P3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="7"/>
+      <c r="Q3" s="7" t="s">
+        <v>19</v>
+      </c>
       <c r="R3" s="7"/>
       <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:19">
-      <c r="A4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="13" t="s">
+    <row r="4" s="2" customFormat="1" spans="1:20">
+      <c r="A4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="14" t="s">
+      <c r="C4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="14" t="s">
+      <c r="I4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="M4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="N4" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="O4" s="14" t="s">
+      <c r="K4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="N4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="P4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="Q4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
+      <c r="R4" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="13"/>
+      <c r="T4" s="13"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:19">
-      <c r="A5" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
+    <row r="5" s="3" customFormat="1" spans="1:20">
+      <c r="A5" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:19">
-      <c r="A6" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
-      <c r="S6" s="16"/>
+    <row r="6" s="3" customFormat="1" spans="1:20">
+      <c r="A6" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="15"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:19">
-      <c r="A7" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:20">
+      <c r="A7" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="17"/>
     </row>
-    <row r="8" spans="1:19">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="19" t="s">
+    <row r="8" spans="1:20">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="C8" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="19"/>
-      <c r="H8" s="5">
+      <c r="F8" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="18"/>
+      <c r="I8" s="5">
         <v>1</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J8" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="L8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="5">
+      <c r="K8" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N8" s="5">
         <v>1</v>
       </c>
-      <c r="N8" s="5">
+      <c r="O8" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:19">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="5">
+    <row r="9" spans="1:20">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="5">
         <v>2</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J9" s="19"/>
-      <c r="L9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M9" s="5">
+      <c r="J9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="18"/>
+      <c r="M9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N9" s="5">
         <v>1</v>
       </c>
-      <c r="N9" s="5">
+      <c r="O9" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="H10" s="5">
+    <row r="10" spans="1:20">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="I10" s="5">
         <v>3</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="L10" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="K10" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="H1:Q1"/>
-    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="I1:R1"/>
+    <mergeCell ref="N2:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>